<commit_message>
Channel files for 7/27 test
</commit_message>
<xml_diff>
--- a/LDC_Dual_log.xlsx
+++ b/LDC_Dual_log.xlsx
@@ -249,80 +249,84 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -431,498 +435,495 @@
   <dimension ref="A1:P25"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.66"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="51" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="I2" s="7" t="n">
+      <c r="I2" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="J2" s="8" t="n">
+      <c r="J2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K2" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="L2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="M2" s="5" t="n">
+      <c r="M2" s="6" t="n">
         <v>-1</v>
       </c>
-      <c r="N2" s="0" t="n">
+      <c r="N2" s="1" t="n">
         <f aca="false">HEX2DEC(K2)+L2</f>
         <v>144</v>
       </c>
-      <c r="O2" s="0" t="n">
+      <c r="O2" s="1" t="n">
         <f aca="false">HEX2DEC(K2)+4</f>
         <v>148</v>
       </c>
-      <c r="P2" s="0" t="n">
+      <c r="P2" s="1" t="n">
         <f aca="false">IF(M2=3,HEX2DEC(K2)+3,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="D3" s="10" t="n">
         <v>36</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="9" t="n">
+      <c r="G3" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="H3" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="I3" s="12" t="n">
+      <c r="I3" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="J3" s="13" t="n">
+      <c r="J3" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="K3" s="9" t="n">
+      <c r="K3" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="L3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="M3" s="5" t="n">
+      <c r="M3" s="6" t="n">
         <v>-1</v>
       </c>
-      <c r="N3" s="0" t="n">
+      <c r="N3" s="1" t="n">
         <f aca="false">HEX2DEC(K3)+L3</f>
         <v>256</v>
       </c>
-      <c r="O3" s="0" t="n">
+      <c r="O3" s="1" t="n">
         <f aca="false">HEX2DEC(K3)+4</f>
         <v>260</v>
       </c>
-      <c r="P3" s="0" t="n">
+      <c r="P3" s="1" t="n">
         <f aca="false">IF(M3=3,HEX2DEC(K3)+3,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="I4" s="7" t="n">
+      <c r="I4" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="1" t="n">
+      <c r="K4" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="L4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="M4" s="6" t="n">
         <v>-1</v>
       </c>
-      <c r="N4" s="0" t="n">
+      <c r="N4" s="1" t="n">
         <f aca="false">HEX2DEC(K4)+L4</f>
         <v>145</v>
       </c>
-      <c r="O4" s="0" t="n">
+      <c r="O4" s="1" t="n">
         <f aca="false">HEX2DEC(K4)+4</f>
         <v>148</v>
       </c>
-      <c r="P4" s="0" t="n">
+      <c r="P4" s="1" t="n">
         <f aca="false">IF(M4=3,HEX2DEC(K4)+3,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="14" t="n">
+      <c r="H5" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="I5" s="17" t="n">
+      <c r="I5" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="K5" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="L5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="M5" s="6" t="n">
         <v>-1</v>
       </c>
-      <c r="N5" s="0" t="n">
+      <c r="N5" s="1" t="n">
         <f aca="false">HEX2DEC(K5)+L5</f>
         <v>257</v>
       </c>
-      <c r="O5" s="0" t="n">
+      <c r="O5" s="1" t="n">
         <f aca="false">HEX2DEC(K5)+4</f>
         <v>260</v>
       </c>
-      <c r="P5" s="0" t="n">
+      <c r="P5" s="1" t="n">
         <f aca="false">IF(M5=3,HEX2DEC(K5)+3,19)</f>
         <v>19</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="P6" s="0" t="n">
-        <f aca="false">IF(M6=3,HEX2DEC(K6)+3,19)</f>
-        <v>19</v>
-      </c>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="P6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="15"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="19"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="6"/>
+      <c r="M18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="7"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G22" s="5"/>
+      <c r="G22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G23" s="5"/>
+      <c r="G23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G24" s="5"/>
+      <c r="G24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="23"/>
-      <c r="G25" s="24"/>
+      <c r="B25" s="24"/>
+      <c r="G25" s="25"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>